<commit_message>
S32: newest veneer file (hộc kéo 23/10 and 24/10)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Loss_time_S32_05-10_den_24-10.xlsx
+++ b/loss-time/outputs/Loss_time_S32_05-10_den_24-10.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Ghi chú review" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'S32 5-10 đến 24-10'!$A$2:$R$56</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'S32 5-10 đến 24-10'!$A$2:$R$57</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="226">
   <si>
     <t xml:space="preserve">LOSS TIME MÃ S32 (OTHER SUPPORT OF PRODUCTION) - 05/10 ĐẾN 24/10/2026 - LÀM RIÊNG, KHÔNG LẪN MÃ KHÁC</t>
   </si>
@@ -389,6 +389,15 @@
     <t xml:space="preserve">Charge to: HÀNG BẢNG MÀU</t>
   </si>
   <si>
+    <t xml:space="preserve">RH12-4706-0423</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sửa hàng hộc kéo (veneer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hàng hộc kéo, 4 người cả ngày</t>
+  </si>
+  <si>
     <t xml:space="preserve">AR15-1016-892</t>
   </si>
   <si>
@@ -413,13 +422,7 @@
     <t xml:space="preserve">code 239 (130 m2)</t>
   </si>
   <si>
-    <t xml:space="preserve">RH12-4706-0423</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sửa hàng hộc kéo (veneer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy 24/10 8:00-20:00 (có thể là giờ dự kiến)</t>
+    <t xml:space="preserve">Hàng hộc kéo, 2 người</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -668,7 +671,7 @@
     <t xml:space="preserve">1. Bảng này CHỈ chứa mã S32, tách hoàn toàn khỏi bảng P20/P26/P22/A2 (không lẫn mã khác). Khi bạn cập nhật, tôi giữ nguyên nguyên tắc này.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Nguồn: 5 file trong gói zip (lấy bản mới nhất mỗi loại: Beam saw bản 24/10, UV bản (1), Ép nóng bản (1), Veneer bản 24/10, file sửa hàng MAC Mr.Hiệp) và 3 hình (thợ sơn tuần 42, cào cước 16/10, bắn cát 15/10). Chỉ lấy dòng từ 05/10 đến 24/10. UV (báo cáo ngày đến 11/10, phát sinh đến 13/10) và Ép nóng (đến 6/10) chưa có số liệu mới.</t>
+    <t xml:space="preserve">2. Nguồn: 5 file trong gói zip (lấy bản mới nhất mỗi loại: Beam saw bản 24/10, UV bản (1), Ép nóng bản (1), Veneer bản mới nhất 24/10, file sửa hàng MAC Mr.Hiệp) và 3 hình (thợ sơn tuần 42, cào cước 16/10, bắn cát 15/10). Chỉ lấy dòng từ 05/10 đến 24/10. UV (báo cáo ngày đến 11/10, phát sinh đến 13/10) và Ép nóng (đến 6/10) chưa có số liệu mới.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Tất cả giờ công trong bảng khớp với số giờ trong nguồn (sheet "Đối chiếu nguồn"). Tổng giờ công xem sheet "Đối chiếu nguồn".</t>
@@ -701,7 +704,7 @@
     <t xml:space="preserve">12. File sửa hàng MAC (Mr.Hiệp) là nguồn mới: 14/10 (AR1069F1233, chạy nhỏ lại mộng, 2 người, 9:00-10:00) và 23/10 (AR15-1016-892, khoan lại lỗ vít 11mm, 2 người, 9:32-11:20). Khu vực Machining, bộ phận ME (cột "Hỗ trợ sửa"). Dòng 23/10: cột tổng thời gian ghi 1:55 nhưng 9:32-11:20 là 1:48, bảng lấy theo giờ bắt đầu - kết thúc (3,6 giờ công) nên sheet Đối chiếu nguồn lệch 0,23 giờ (tô vàng).</t>
   </si>
   <si>
-    <t xml:space="preserve">13. Veneer 24/10 (Thứ Bảy): soạn hàng veneer lỗi trả lại kho (2 người 8:00-9:30, 3 giờ, ME) và sửa hàng hộc kéo RH12-4706-0423 (4 người 8:00-20:00, 48 giờ, ME). Dòng 48 giờ có thể là giờ dự kiến (tô vàng).</t>
+    <t xml:space="preserve">13. Veneer 23/10 và 24/10: sửa hàng hộc kéo RH12-4706-0423: 23/10 4 người 8:00-20:00 (48 giờ, ME; bản trước ghi nhầm ngày 24/10, bản mới đã đổi sang 23/10) và 24/10 2 người 8:00-15:00 (14 giờ, ME, thêm mới). Veneer 24/10 còn dòng soạn hàng veneer lỗi trả lại kho (2 người 8:00-9:30, 3 giờ, ME).</t>
   </si>
   <si>
     <t xml:space="preserve">14. Beam saw 22/10: 7 dòng "HÀNG BẢNG MÀU" (W0114F08, W0276F03, W1981F1055, W2629F1222, W0164F01 x2, W2446F1200) chưa có giờ bắt đầu/kết thúc trong nguồn nên chưa đưa vào bảng (0 giờ). Cần hỏi giờ nếu muốn nhập. Hàng bảng màu theo tiền lệ ghi bộ phận TECHNICAL FINISHING.</t>
@@ -1395,7 +1398,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -4144,240 +4147,295 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13" t="str">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B53,21)</f>
         <v>W43</v>
       </c>
-      <c r="B53" s="14" t="n">
+      <c r="B53" s="4" t="n">
         <v>46318</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C53" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13" t="n">
-        <v>65</v>
-      </c>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H53" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I53" s="15" t="s">
+      <c r="D53" s="3"/>
+      <c r="E53" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I53" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J53" s="13" t="s">
+      <c r="J53" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K53" s="15" t="s">
+      <c r="K53" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L53" s="15" t="s">
+      <c r="L53" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="M53" s="16" t="n">
-        <v>0.397222222222222</v>
-      </c>
-      <c r="N53" s="16" t="n">
-        <v>0.472222222222222</v>
-      </c>
-      <c r="O53" s="17" t="n">
+      <c r="M53" s="6" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="N53" s="6" t="n">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="O53" s="7" t="n">
         <f aca="false">(N53-M53)*24</f>
-        <v>1.8</v>
-      </c>
-      <c r="P53" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q53" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="P53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q53" s="7" t="n">
         <f aca="false">P53*O53</f>
-        <v>3.6</v>
-      </c>
-      <c r="R53" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8" t="str">
+        <v>48</v>
+      </c>
+      <c r="R53" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="13" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B54,21)</f>
         <v>W43</v>
       </c>
-      <c r="B54" s="9" t="n">
-        <v>46319</v>
-      </c>
-      <c r="C54" s="10" t="s">
+      <c r="B54" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C54" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H54" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I54" s="10" t="s">
+      <c r="D54" s="13"/>
+      <c r="E54" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H54" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I54" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="J54" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="K54" s="10" t="s">
+      <c r="J54" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="K54" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="L54" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="M54" s="11" t="n">
-        <v>0.416666666666667</v>
-      </c>
-      <c r="N54" s="11" t="n">
-        <v>0.420833333333333</v>
-      </c>
-      <c r="O54" s="12" t="n">
+      <c r="L54" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="M54" s="16" t="n">
+        <v>0.397222222222222</v>
+      </c>
+      <c r="N54" s="16" t="n">
+        <v>0.472222222222222</v>
+      </c>
+      <c r="O54" s="17" t="n">
         <f aca="false">(N54-M54)*24</f>
-        <v>0.1</v>
-      </c>
-      <c r="P54" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q54" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="P54" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q54" s="17" t="n">
         <f aca="false">P54*O54</f>
-        <v>0.3</v>
-      </c>
-      <c r="R54" s="8" t="s">
-        <v>41</v>
+        <v>3.6</v>
+      </c>
+      <c r="R54" s="13" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="str">
+      <c r="A55" s="8" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B55,21)</f>
         <v>W43</v>
       </c>
-      <c r="B55" s="4" t="n">
+      <c r="B55" s="9" t="n">
         <v>46319</v>
       </c>
-      <c r="C55" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I55" s="5" t="s">
+      <c r="C55" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F55" s="8"/>
+      <c r="G55" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H55" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I55" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J55" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="L55" s="5" t="s">
+      <c r="J55" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="K55" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="M55" s="6" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="N55" s="6" t="n">
-        <v>0.395833333333333</v>
-      </c>
-      <c r="O55" s="7" t="n">
+      <c r="L55" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="M55" s="11" t="n">
+        <v>0.416666666666667</v>
+      </c>
+      <c r="N55" s="11" t="n">
+        <v>0.420833333333333</v>
+      </c>
+      <c r="O55" s="12" t="n">
         <f aca="false">(N55-M55)*24</f>
-        <v>1.5</v>
-      </c>
-      <c r="P55" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q55" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="P55" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q55" s="12" t="n">
         <f aca="false">P55*O55</f>
-        <v>3</v>
-      </c>
-      <c r="R55" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="13" t="str">
+        <v>0.3</v>
+      </c>
+      <c r="R55" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B56,21)</f>
         <v>W43</v>
       </c>
-      <c r="B56" s="14" t="n">
+      <c r="B56" s="4" t="n">
         <v>46319</v>
       </c>
-      <c r="C56" s="15" t="s">
+      <c r="C56" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="F56" s="13"/>
-      <c r="G56" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H56" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I56" s="15" t="s">
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I56" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J56" s="13" t="s">
+      <c r="J56" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K56" s="15" t="s">
+      <c r="K56" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="L56" s="15" t="s">
+      <c r="L56" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="M56" s="16" t="n">
+      <c r="M56" s="6" t="n">
         <v>0.333333333333333</v>
       </c>
-      <c r="N56" s="16" t="n">
-        <v>0.833333333333333</v>
-      </c>
-      <c r="O56" s="17" t="n">
+      <c r="N56" s="6" t="n">
+        <v>0.395833333333333</v>
+      </c>
+      <c r="O56" s="7" t="n">
         <f aca="false">(N56-M56)*24</f>
-        <v>12</v>
-      </c>
-      <c r="P56" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q56" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q56" s="7" t="n">
         <f aca="false">P56*O56</f>
-        <v>48</v>
-      </c>
-      <c r="R56" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="R56" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P57" s="18" t="s">
+      <c r="A57" s="3" t="str">
+        <f aca="false">"W"&amp;WEEKNUM(B57,21)</f>
+        <v>W43</v>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L57" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="Q57" s="19" t="n">
-        <f aca="false">SUM(Q3:Q56)</f>
-        <v>1826.33333333333</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="20" t="s">
+      <c r="M57" s="6" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="N57" s="6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="O57" s="7" t="n">
+        <f aca="false">(N57-M57)*24</f>
+        <v>7</v>
+      </c>
+      <c r="P57" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <f aca="false">P57*O57</f>
+        <v>14</v>
+      </c>
+      <c r="R57" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P58" s="18" t="s">
         <v>131</v>
       </c>
+      <c r="Q58" s="19" t="n">
+        <f aca="false">SUM(Q3:Q57)</f>
+        <v>1840.33333333333</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="20" t="s">
+        <v>132</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R56"/>
+  <autoFilter ref="A2:R57"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4405,18 +4463,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>26</v>
@@ -4446,7 +4504,7 @@
         <v>85</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4454,46 +4512,46 @@
         <v>46300</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A4,21)</f>
         <v>W41</v>
       </c>
       <c r="D4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>46</v>
       </c>
       <c r="E4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>120</v>
       </c>
       <c r="F4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A4,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A4,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M4" s="24" t="n">
@@ -4506,46 +4564,46 @@
         <v>46301</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C5" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A5,21)</f>
         <v>W41</v>
       </c>
       <c r="D5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>55</v>
       </c>
       <c r="E5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>120</v>
       </c>
       <c r="F5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A5,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A5,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M5" s="24" t="n">
@@ -4558,46 +4616,46 @@
         <v>46302</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C6" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A6,21)</f>
         <v>W41</v>
       </c>
       <c r="D6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>112</v>
       </c>
       <c r="F6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A6,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A6,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M6" s="24" t="n">
@@ -4610,46 +4668,46 @@
         <v>46303</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C7" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A7,21)</f>
         <v>W41</v>
       </c>
       <c r="D7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>104</v>
       </c>
       <c r="F7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.2</v>
       </c>
       <c r="G7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A7,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A7,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M7" s="24" t="n">
@@ -4662,46 +4720,46 @@
         <v>46304</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C8" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A8,21)</f>
         <v>W41</v>
       </c>
       <c r="D8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>132</v>
       </c>
       <c r="F8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.6</v>
       </c>
       <c r="G8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A8,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A8,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M8" s="24" t="n">
@@ -4714,46 +4772,46 @@
         <v>46305</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C9" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A9,21)</f>
         <v>W41</v>
       </c>
       <c r="D9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>116</v>
       </c>
       <c r="F9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>3</v>
       </c>
       <c r="H9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A9,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A9,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M9" s="24" t="n">
@@ -4766,46 +4824,46 @@
         <v>46306</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C10" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A10,21)</f>
         <v>W41</v>
       </c>
       <c r="D10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>72</v>
       </c>
       <c r="F10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A10,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A10,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M10" s="24" t="n">
@@ -4818,46 +4876,46 @@
         <v>46307</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C11" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A11,21)</f>
         <v>W42</v>
       </c>
       <c r="D11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>18</v>
       </c>
       <c r="J11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>144</v>
       </c>
       <c r="K11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A11,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A11,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M11" s="24" t="n">
@@ -4870,46 +4928,46 @@
         <v>46308</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C12" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A12,21)</f>
         <v>W42</v>
       </c>
       <c r="D12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>4.5</v>
       </c>
       <c r="J12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>144</v>
       </c>
       <c r="K12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A12,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A12,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M12" s="24" t="n">
@@ -4922,46 +4980,46 @@
         <v>46309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A13,21)</f>
         <v>W42</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>2</v>
       </c>
       <c r="I13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>144</v>
       </c>
       <c r="K13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A13,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A13,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M13" s="24" t="n">
@@ -4974,46 +5032,46 @@
         <v>46310</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C14" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A14,21)</f>
         <v>W42</v>
       </c>
       <c r="D14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0.333333333333333</v>
       </c>
       <c r="H14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>144</v>
       </c>
       <c r="K14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A14,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A14,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>32</v>
       </c>
       <c r="M14" s="24" t="n">
@@ -5026,46 +5084,46 @@
         <v>46311</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C15" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A15,21)</f>
         <v>W42</v>
       </c>
       <c r="D15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.75</v>
       </c>
       <c r="G15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>144</v>
       </c>
       <c r="K15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>9</v>
       </c>
       <c r="L15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A15,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A15,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M15" s="24" t="n">
@@ -5078,46 +5136,46 @@
         <v>46312</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C16" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A16,21)</f>
         <v>W42</v>
       </c>
       <c r="D16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.2</v>
       </c>
       <c r="G16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>96</v>
       </c>
       <c r="K16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A16,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A16,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M16" s="24" t="n">
@@ -5130,46 +5188,46 @@
         <v>46314</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C17" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A17,21)</f>
         <v>W43</v>
       </c>
       <c r="D17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.35</v>
       </c>
       <c r="G17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A17,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A17,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M17" s="24" t="n">
@@ -5182,46 +5240,46 @@
         <v>46315</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C18" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A18,21)</f>
         <v>W43</v>
       </c>
       <c r="D18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.4</v>
       </c>
       <c r="G18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>4</v>
       </c>
       <c r="H18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A18,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A18,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M18" s="24" t="n">
@@ -5234,46 +5292,46 @@
         <v>46317</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C19" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A19,21)</f>
         <v>W43</v>
       </c>
       <c r="D19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>3.1</v>
       </c>
       <c r="G19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
         <v>0</v>
       </c>
       <c r="H19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A19,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A19,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M19" s="24" t="n">
@@ -5286,51 +5344,51 @@
         <v>46318</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C20" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A20,21)</f>
         <v>W43</v>
       </c>
       <c r="D20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0</v>
       </c>
       <c r="G20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
+        <v>48</v>
       </c>
       <c r="H20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>3.6</v>
       </c>
       <c r="I20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A20,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A20,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M20" s="24" t="n">
         <f aca="false">SUM(D20:L20)</f>
-        <v>3.6</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5338,56 +5396,56 @@
         <v>46319</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C21" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A21,21)</f>
         <v>W43</v>
       </c>
       <c r="D21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,D$3)</f>
         <v>0</v>
       </c>
       <c r="E21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,E$3)</f>
         <v>0</v>
       </c>
       <c r="F21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,F$3)</f>
         <v>0.3</v>
       </c>
       <c r="G21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,G$3)</f>
-        <v>51</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,G$3)</f>
+        <v>17</v>
       </c>
       <c r="H21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,H$3)</f>
         <v>0</v>
       </c>
       <c r="I21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,I$3)</f>
         <v>0</v>
       </c>
       <c r="J21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,J$3)</f>
         <v>0</v>
       </c>
       <c r="K21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,K$3)</f>
         <v>0</v>
       </c>
       <c r="L21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$B$3:$B$56,$A21,'S32 5-10 đến 24-10'!$R$3:$R$56,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$B$3:$B$57,$A21,'S32 5-10 đến 24-10'!$R$3:$R$57,L$3)</f>
         <v>0</v>
       </c>
       <c r="M21" s="24" t="n">
         <f aca="false">SUM(D21:L21)</f>
-        <v>51.3</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B22" s="25"/>
       <c r="C22" s="25"/>
@@ -5405,7 +5463,7 @@
       </c>
       <c r="G22" s="24" t="n">
         <f aca="false">SUM(G4:G21)</f>
-        <v>58.3333333333333</v>
+        <v>72.3333333333333</v>
       </c>
       <c r="H22" s="24" t="n">
         <f aca="false">SUM(H4:H21)</f>
@@ -5429,47 +5487,47 @@
       </c>
       <c r="M22" s="24" t="n">
         <f aca="false">SUM(M4:M21)</f>
-        <v>1826.33333333333</v>
+        <v>1840.33333333333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B26" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$A$3:$A$56,A26)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$A$3:$A$57,A26)</f>
         <v>880.8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B27" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$A$3:$A$56,A27)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$A$3:$A$57,A27)</f>
         <v>882.783333333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B28" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$A$3:$A$56,A28)</f>
-        <v>62.75</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$A$3:$A$57,A28)</f>
+        <v>76.75</v>
       </c>
     </row>
   </sheetData>
@@ -5488,7 +5546,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -5506,19 +5564,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>13</v>
@@ -5527,19 +5585,19 @@
         <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I1" s="28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J1" s="28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K1" s="28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L1" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7358,149 +7416,149 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="40" t="n">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="29" t="n">
         <v>46318</v>
       </c>
-      <c r="B52" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="C52" s="42" t="s">
+      <c r="B52" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="D52" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="E52" s="41" t="s">
+      <c r="D52" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E52" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="F52" s="43" t="n">
-        <v>0.397222222222222</v>
-      </c>
-      <c r="G52" s="43" t="n">
-        <v>0.472222222222222</v>
-      </c>
-      <c r="H52" s="41" t="n">
-        <v>2</v>
+      <c r="F52" s="32" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G52" s="32" t="n">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="H52" s="30" t="n">
+        <v>4</v>
       </c>
       <c r="I52" s="33" t="s">
         <v>119</v>
       </c>
       <c r="J52" s="34" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="K52" s="35" t="s">
         <v>121</v>
       </c>
       <c r="L52" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="36" t="n">
-        <v>46319</v>
-      </c>
-      <c r="B53" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="C53" s="38" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="40" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B53" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="D53" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="E53" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="F53" s="39" t="n">
-        <v>0.416666666666667</v>
-      </c>
-      <c r="G53" s="39" t="n">
-        <v>0.420833333333333</v>
-      </c>
-      <c r="H53" s="37" t="n">
-        <v>3</v>
+      <c r="D53" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E53" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="F53" s="43" t="n">
+        <v>0.397222222222222</v>
+      </c>
+      <c r="G53" s="43" t="n">
+        <v>0.472222222222222</v>
+      </c>
+      <c r="H53" s="41" t="n">
+        <v>2</v>
       </c>
       <c r="I53" s="33" t="s">
         <v>122</v>
       </c>
       <c r="J53" s="34" t="n">
+        <v>65</v>
+      </c>
+      <c r="K53" s="35" t="s">
+        <v>124</v>
+      </c>
+      <c r="L53" s="34" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="36" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B54" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="D54" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="F54" s="39" t="n">
+        <v>0.416666666666667</v>
+      </c>
+      <c r="G54" s="39" t="n">
+        <v>0.420833333333333</v>
+      </c>
+      <c r="H54" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="I54" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="J54" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="K53" s="35" t="s">
+      <c r="K54" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="L53" s="34" t="s">
+      <c r="L54" s="34" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="29" t="n">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="29" t="n">
         <v>46319</v>
       </c>
-      <c r="B54" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="D54" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E54" s="30" t="s">
+      <c r="B55" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="D55" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E55" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="F54" s="32" t="n">
+      <c r="F55" s="32" t="n">
         <v>0.333333333333333</v>
       </c>
-      <c r="G54" s="32" t="n">
+      <c r="G55" s="32" t="n">
         <v>0.395833333333333</v>
       </c>
-      <c r="H54" s="30" t="n">
+      <c r="H55" s="30" t="n">
         <v>2</v>
-      </c>
-      <c r="I54" s="33" t="s">
-        <v>124</v>
-      </c>
-      <c r="J54" s="34"/>
-      <c r="K54" s="35" t="s">
-        <v>126</v>
-      </c>
-      <c r="L54" s="34" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="40" t="n">
-        <v>46319</v>
-      </c>
-      <c r="B55" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="C55" s="42" t="s">
-        <v>128</v>
-      </c>
-      <c r="D55" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="E55" s="41" t="s">
-        <v>76</v>
-      </c>
-      <c r="F55" s="43" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="G55" s="43" t="n">
-        <v>0.833333333333333</v>
-      </c>
-      <c r="H55" s="41" t="n">
-        <v>4</v>
       </c>
       <c r="I55" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="J55" s="34" t="n">
-        <v>30</v>
-      </c>
+      <c r="J55" s="34"/>
       <c r="K55" s="35" t="s">
         <v>129</v>
       </c>
@@ -7508,9 +7566,47 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="20" t="s">
-        <v>159</v>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="29" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B56" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="D56" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="F56" s="32" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G56" s="32" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="H56" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I56" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="J56" s="34" t="n">
+        <v>22</v>
+      </c>
+      <c r="K56" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="L56" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="20" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -7541,7 +7637,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7549,16 +7645,16 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7569,7 +7665,7 @@
         <v>5.9</v>
       </c>
       <c r="C4" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A4)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A4)</f>
         <v>5.9</v>
       </c>
       <c r="D4" s="46" t="n">
@@ -7589,7 +7685,7 @@
         <v>776</v>
       </c>
       <c r="C5" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A5)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A5)</f>
         <v>776</v>
       </c>
       <c r="D5" s="46" t="n">
@@ -7609,7 +7705,7 @@
         <v>22.5</v>
       </c>
       <c r="C6" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A6)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A6)</f>
         <v>22.5</v>
       </c>
       <c r="D6" s="46" t="n">
@@ -7629,7 +7725,7 @@
         <v>101</v>
       </c>
       <c r="C7" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A7)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A7)</f>
         <v>101</v>
       </c>
       <c r="D7" s="46" t="n">
@@ -7646,11 +7742,11 @@
         <v>62</v>
       </c>
       <c r="B8" s="45" t="n">
-        <v>58.3333</v>
+        <v>72.3333</v>
       </c>
       <c r="C8" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A8)</f>
-        <v>58.3333333333333</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A8)</f>
+        <v>72.3333333333333</v>
       </c>
       <c r="D8" s="46" t="n">
         <f aca="false">C8-B8</f>
@@ -7669,7 +7765,7 @@
         <v>5.8333</v>
       </c>
       <c r="C9" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A9)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A9)</f>
         <v>5.6</v>
       </c>
       <c r="D9" s="46" t="n">
@@ -7689,7 +7785,7 @@
         <v>816</v>
       </c>
       <c r="C10" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A10)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A10)</f>
         <v>816</v>
       </c>
       <c r="D10" s="46" t="n">
@@ -7709,7 +7805,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A11)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A11)</f>
         <v>9</v>
       </c>
       <c r="D11" s="46" t="n">
@@ -7729,7 +7825,7 @@
         <v>32</v>
       </c>
       <c r="C12" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$56,'S32 5-10 đến 24-10'!$R$3:$R$56,A12)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 24-10'!$Q$3:$Q$57,'S32 5-10 đến 24-10'!$R$3:$R$57,A12)</f>
         <v>32</v>
       </c>
       <c r="D12" s="46" t="n">
@@ -7743,15 +7839,15 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="47" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B13" s="48" t="n">
         <f aca="false">SUM(B4:B12)</f>
-        <v>1826.5666</v>
+        <v>1840.5666</v>
       </c>
       <c r="C13" s="48" t="n">
         <f aca="false">SUM(C4:C12)</f>
-        <v>1826.33333333333</v>
+        <v>1840.33333333333</v>
       </c>
       <c r="D13" s="48" t="n">
         <f aca="false">SUM(D4:D12)</f>
@@ -7764,7 +7860,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -7795,19 +7891,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7818,10 +7914,10 @@
         <v>26</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E2" s="26" t="n">
         <v>10</v>
@@ -7835,10 +7931,10 @@
         <v>26</v>
       </c>
       <c r="C3" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="D3" s="26" t="s">
         <v>171</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>170</v>
       </c>
       <c r="E3" s="26" t="n">
         <v>5</v>
@@ -7852,10 +7948,10 @@
         <v>26</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>10</v>
@@ -7869,10 +7965,10 @@
         <v>26</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E5" s="26" t="n">
         <v>27</v>
@@ -7886,10 +7982,10 @@
         <v>26</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>23</v>
@@ -7903,10 +7999,10 @@
         <v>26</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>27</v>
@@ -7920,10 +8016,10 @@
         <v>26</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>23</v>
@@ -7937,10 +8033,10 @@
         <v>62</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E9" s="26" t="n">
         <v>50</v>
@@ -7954,10 +8050,10 @@
         <v>62</v>
       </c>
       <c r="C10" s="26" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" s="26" t="s">
         <v>179</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>178</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>100</v>
@@ -7971,10 +8067,10 @@
         <v>65</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E11" s="26" t="n">
         <v>13</v>
@@ -7988,10 +8084,10 @@
         <v>65</v>
       </c>
       <c r="C12" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="D12" s="26" t="s">
         <v>182</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>181</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>13</v>
@@ -8005,10 +8101,10 @@
         <v>65</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E13" s="26" t="n">
         <v>13</v>
@@ -8022,10 +8118,10 @@
         <v>65</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>13</v>
@@ -8039,10 +8135,10 @@
         <v>65</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E15" s="26" t="n">
         <v>13</v>
@@ -8056,10 +8152,10 @@
         <v>65</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>13</v>
@@ -8073,10 +8169,10 @@
         <v>65</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E17" s="26" t="n">
         <v>13</v>
@@ -8090,10 +8186,10 @@
         <v>65</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>13</v>
@@ -8107,10 +8203,10 @@
         <v>65</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E19" s="26" t="n">
         <v>13</v>
@@ -8124,10 +8220,10 @@
         <v>65</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E20" s="26" t="n">
         <v>13</v>
@@ -8141,10 +8237,10 @@
         <v>65</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E21" s="26" t="n">
         <v>13</v>
@@ -8158,10 +8254,10 @@
         <v>65</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E22" s="26" t="n">
         <v>13</v>
@@ -8175,10 +8271,10 @@
         <v>65</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E23" s="26" t="n">
         <v>13</v>
@@ -8192,10 +8288,10 @@
         <v>65</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E24" s="26" t="n">
         <v>13</v>
@@ -8209,10 +8305,10 @@
         <v>65</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E25" s="26" t="n">
         <v>455</v>
@@ -8226,10 +8322,10 @@
         <v>65</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E26" s="26" t="n">
         <v>299</v>
@@ -8243,10 +8339,10 @@
         <v>65</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E27" s="26" t="n">
         <v>286</v>
@@ -8260,10 +8356,10 @@
         <v>65</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E28" s="26" t="n">
         <v>1092</v>
@@ -8277,10 +8373,10 @@
         <v>65</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E29" s="26" t="n">
         <v>156</v>
@@ -8294,10 +8390,10 @@
         <v>65</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E30" s="26" t="n">
         <v>13</v>
@@ -8311,10 +8407,10 @@
         <v>65</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E31" s="26" t="n">
         <v>13</v>
@@ -8328,10 +8424,10 @@
         <v>65</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E32" s="26" t="n">
         <v>13</v>
@@ -8345,10 +8441,10 @@
         <v>65</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E33" s="26" t="n">
         <v>13</v>
@@ -8365,7 +8461,7 @@
         <v>74</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E34" s="26" t="n">
         <v>100</v>
@@ -8382,7 +8478,7 @@
         <v>80</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E35" s="26" t="n">
         <v>4</v>
@@ -8399,7 +8495,7 @@
         <v>109</v>
       </c>
       <c r="D36" s="26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E36" s="26" t="n">
         <v>30</v>
@@ -8416,7 +8512,7 @@
         <v>110</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E37" s="26" t="n">
         <v>2</v>
@@ -8433,7 +8529,7 @@
         <v>114</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E38" s="26" t="n">
         <v>30</v>
@@ -8447,10 +8543,10 @@
         <v>79</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D39" s="26" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E39" s="26" t="n">
         <v>65</v>
@@ -8464,13 +8560,13 @@
         <v>62</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D40" s="26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E40" s="26" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -8497,77 +8593,77 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="51" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="51" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>